<commit_message>
Improve batch preparation, manual review and English documentation
</commit_message>
<xml_diff>
--- a/examples/lab_forms_excel/xlsx/plantar.xlsx
+++ b/examples/lab_forms_excel/xlsx/plantar.xlsx
@@ -31,7 +31,7 @@
           <x:t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Источник: photo_4_plantar_pretest3_2026-07-14.xlsx</x:t>
+    Source: photo_4_plantar_pretest3_2026-07-14.xlsx</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -41,7 +41,7 @@
           <x:t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Порядковый номер. Формула ROW()-6 пересчитывает нумерацию при вставке и удалении строк данных.</x:t>
+    Sequential ID. The ROW()-6 formula updates numbering when data rows are inserted or deleted.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -51,7 +51,7 @@
           <x:t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    L1: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</x:t>
+    L1: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -61,7 +61,7 @@
           <x:t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    L2: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</x:t>
+    L2: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -71,7 +71,7 @@
           <x:t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    L3: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</x:t>
+    L3: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -81,7 +81,7 @@
           <x:t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    L4: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</x:t>
+    L4: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -91,7 +91,7 @@
           <x:t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    L5: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</x:t>
+    L5: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -101,7 +101,7 @@
           <x:t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    R1: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</x:t>
+    R1: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -111,7 +111,7 @@
           <x:t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    R2: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</x:t>
+    R2: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -121,7 +121,7 @@
           <x:t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    R3: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</x:t>
+    R3: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -131,7 +131,7 @@
           <x:t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    R4: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</x:t>
+    R4: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -141,7 +141,7 @@
           <x:t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    R5: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</x:t>
+    R5: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -151,7 +151,7 @@
           <x:t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Примечание к животному; переносится как текст.</x:t>
+    Animal notes; recognized and exported as text.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -524,43 +524,43 @@
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
   <xltc:threadedComment ref="A1" dT="2026-09-14T15:06:57.547" personId="{B425DE92-BFBD-455F-8ACE-961BDAB0B5C7}" id="{95E57A52-E21D-49F4-BCBB-FD885B92565D}">
-    <xltc:text>Источник: photo_4_plantar_pretest3_2026-07-14.xlsx</xltc:text>
+    <xltc:text>Source: photo_4_plantar_pretest3_2026-07-14.xlsx</xltc:text>
   </xltc:threadedComment>
   <xltc:threadedComment ref="A6" dT="2026-09-14T15:06:57.547" personId="{B425DE92-BFBD-455F-8ACE-961BDAB0B5C7}" id="{7E198E70-76D5-477E-9BC0-F02E78DC8B3E}">
-    <xltc:text>Порядковый номер. Формула ROW()-6 пересчитывает нумерацию при вставке и удалении строк данных.</xltc:text>
+    <xltc:text>Sequential ID. The ROW()-6 formula updates numbering when data rows are inserted or deleted.</xltc:text>
   </xltc:threadedComment>
   <xltc:threadedComment ref="B6" dT="2026-09-14T15:06:57.547" personId="{B425DE92-BFBD-455F-8ACE-961BDAB0B5C7}" id="{2BB9EF0D-B28B-4540-92A9-842AB15BB924}">
-    <xltc:text>L1: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</xltc:text>
+    <xltc:text>L1: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</xltc:text>
   </xltc:threadedComment>
   <xltc:threadedComment ref="C6" dT="2026-09-14T15:06:57.547" personId="{B425DE92-BFBD-455F-8ACE-961BDAB0B5C7}" id="{D62184AA-88C1-4ECB-A0BD-0891D8D89FB3}">
-    <xltc:text>L2: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</xltc:text>
+    <xltc:text>L2: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</xltc:text>
   </xltc:threadedComment>
   <xltc:threadedComment ref="D6" dT="2026-09-14T15:06:57.547" personId="{B425DE92-BFBD-455F-8ACE-961BDAB0B5C7}" id="{C2287B28-B146-4551-86FE-13E25228AE0E}">
-    <xltc:text>L3: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</xltc:text>
+    <xltc:text>L3: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</xltc:text>
   </xltc:threadedComment>
   <xltc:threadedComment ref="E6" dT="2026-09-14T15:06:57.547" personId="{B425DE92-BFBD-455F-8ACE-961BDAB0B5C7}" id="{D268E280-C847-4118-8F04-EF7BEA6A93FB}">
-    <xltc:text>L4: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</xltc:text>
+    <xltc:text>L4: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</xltc:text>
   </xltc:threadedComment>
   <xltc:threadedComment ref="F6" dT="2026-09-14T15:06:57.547" personId="{B425DE92-BFBD-455F-8ACE-961BDAB0B5C7}" id="{9023BB59-D0CA-4804-A401-84BBEAD202FB}">
-    <xltc:text>L5: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</xltc:text>
+    <xltc:text>L5: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</xltc:text>
   </xltc:threadedComment>
   <xltc:threadedComment ref="G6" dT="2026-09-14T15:06:57.547" personId="{B425DE92-BFBD-455F-8ACE-961BDAB0B5C7}" id="{BBF23496-A979-4DAE-900E-44836F3969BD}">
-    <xltc:text>R1: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</xltc:text>
+    <xltc:text>R1: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</xltc:text>
   </xltc:threadedComment>
   <xltc:threadedComment ref="H6" dT="2026-09-14T15:06:57.547" personId="{B425DE92-BFBD-455F-8ACE-961BDAB0B5C7}" id="{B1E53955-7046-4945-B67D-B3A8B10C7DCA}">
-    <xltc:text>R2: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</xltc:text>
+    <xltc:text>R2: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</xltc:text>
   </xltc:threadedComment>
   <xltc:threadedComment ref="I6" dT="2026-09-14T15:06:57.547" personId="{B425DE92-BFBD-455F-8ACE-961BDAB0B5C7}" id="{0F6FD458-6F5C-436B-A59C-C20E7FC20B57}">
-    <xltc:text>R3: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</xltc:text>
+    <xltc:text>R3: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</xltc:text>
   </xltc:threadedComment>
   <xltc:threadedComment ref="J6" dT="2026-09-14T15:06:57.547" personId="{B425DE92-BFBD-455F-8ACE-961BDAB0B5C7}" id="{D4C82D69-41FB-4112-A336-1E959AFC68DD}">
-    <xltc:text>R4: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</xltc:text>
+    <xltc:text>R4: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</xltc:text>
   </xltc:threadedComment>
   <xltc:threadedComment ref="K6" dT="2026-09-14T15:06:57.547" personId="{B425DE92-BFBD-455F-8ACE-961BDAB0B5C7}" id="{E82F6BD1-90E0-4943-9F3E-3B50C72A69DA}">
-    <xltc:text>R5: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</xltc:text>
+    <xltc:text>R5: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</xltc:text>
   </xltc:threadedComment>
   <xltc:threadedComment ref="L6" dT="2026-09-14T15:06:57.547" personId="{B425DE92-BFBD-455F-8ACE-961BDAB0B5C7}" id="{3EF98C35-30F7-4075-A839-EC8649223C9E}">
-    <xltc:text>Примечание к животному; переносится как текст.</xltc:text>
+    <xltc:text>Animal notes; recognized and exported as text.</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
 </file>

</xml_diff>

<commit_message>
Frame metadata fields and limit operator area through R3
</commit_message>
<xml_diff>
--- a/examples/lab_forms_excel/xlsx/plantar.xlsx
+++ b/examples/lab_forms_excel/xlsx/plantar.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plantar" sheetId="1" r:id="Rb922279b074a45aa"/>
-  </x:sheets>
-</x:workbook>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheets>
+    <sheet name="Plantar" sheetId="1" ns1:id="Rdcb5e1c81732420c"/>
+  </sheets>
+</workbook>
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -31,7 +31,7 @@
           <x:t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Source: photo_4_plantar_pretest3_2026-07-14.xlsx</x:t>
+    Источник: photo_4_plantar_pretest3_2026-07-14.xlsx</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -41,7 +41,7 @@
           <x:t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Sequential ID. The ROW()-6 formula updates numbering when data rows are inserted or deleted.</x:t>
+    Порядковый номер. Формула ROW()-6 пересчитывает нумерацию при вставке и удалении строк данных.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -51,7 +51,7 @@
           <x:t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    L1: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</x:t>
+    L1: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -61,7 +61,7 @@
           <x:t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    L2: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</x:t>
+    L2: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -71,7 +71,7 @@
           <x:t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    L3: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</x:t>
+    L3: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -81,7 +81,7 @@
           <x:t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    L4: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</x:t>
+    L4: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -91,7 +91,7 @@
           <x:t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    L5: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</x:t>
+    L5: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -101,7 +101,7 @@
           <x:t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    R1: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</x:t>
+    R1: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -111,7 +111,7 @@
           <x:t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    R2: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</x:t>
+    R2: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -121,7 +121,7 @@
           <x:t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    R3: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</x:t>
+    R3: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -131,7 +131,7 @@
           <x:t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    R4: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</x:t>
+    R4: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -141,7 +141,7 @@
           <x:t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    R5: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</x:t>
+    R5: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -151,7 +151,7 @@
           <x:t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Animal notes; recognized and exported as text.</x:t>
+    Примечание к животному; переносится как текст.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -220,7 +220,7 @@
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="3">
+  <x:borders count="15">
     <x:border/>
     <x:border>
       <x:bottom style="thin">
@@ -241,11 +241,75 @@
         <x:color rgb="FF333333"/>
       </x:bottom>
     </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:top style="none"/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:top style="none"/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:right style="none"/>
+      <x:top style="none"/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="none"/>
+      <x:bottom style="none"/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:bottom style="none"/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:right style="none"/>
+      <x:bottom style="none"/>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="thin">
+        <x:color rgb="FF000000"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FF000000"/>
+      </x:top>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:top style="thin">
+        <x:color rgb="FF000000"/>
+      </x:top>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:right style="thin">
+        <x:color rgb="FF000000"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF000000"/>
+      </x:top>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="thin">
+        <x:color rgb="FF000000"/>
+      </x:left>
+      <x:bottom style="thin">
+        <x:color rgb="FF000000"/>
+      </x:bottom>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:bottom style="thin">
+        <x:color rgb="FF000000"/>
+      </x:bottom>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:right style="thin">
+        <x:color rgb="FF000000"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FF000000"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="21">
+  <x:cellXfs count="34">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -295,6 +359,19 @@
     <x:xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -309,25 +386,25 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Animals_plantar" displayName="Animals_plantar" ref="A6:L26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <tableColumns count="12">
-    <tableColumn id="1" name="ID">
-      <calculatedColumnFormula>ROW()-6</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="2" name="L1"/>
-    <tableColumn id="3" name="L2"/>
-    <tableColumn id="4" name="L3"/>
-    <tableColumn id="5" name="L4"/>
-    <tableColumn id="6" name="L5"/>
-    <tableColumn id="7" name="R1"/>
-    <tableColumn id="8" name="R2"/>
-    <tableColumn id="9" name="R3"/>
-    <tableColumn id="10" name="R4"/>
-    <tableColumn id="11" name="R5"/>
-    <tableColumn id="12" name="Notes"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
-</table>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Animals_plantar" displayName="Animals_plantar" ref="A6:L26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="12">
+    <x:tableColumn id="1" name="ID">
+      <x:calculatedColumnFormula>ROW()-6</x:calculatedColumnFormula>
+    </x:tableColumn>
+    <x:tableColumn id="2" name="L1"/>
+    <x:tableColumn id="3" name="L2"/>
+    <x:tableColumn id="4" name="L3"/>
+    <x:tableColumn id="5" name="L4"/>
+    <x:tableColumn id="6" name="L5"/>
+    <x:tableColumn id="7" name="R1"/>
+    <x:tableColumn id="8" name="R2"/>
+    <x:tableColumn id="9" name="R3"/>
+    <x:tableColumn id="10" name="R4"/>
+    <x:tableColumn id="11" name="R5"/>
+    <x:tableColumn id="12" name="Notes"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
+</x:table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -524,49 +601,49 @@
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
   <xltc:threadedComment ref="A1" dT="2026-09-14T15:06:57.547" personId="{B425DE92-BFBD-455F-8ACE-961BDAB0B5C7}" id="{95E57A52-E21D-49F4-BCBB-FD885B92565D}">
-    <xltc:text>Source: photo_4_plantar_pretest3_2026-07-14.xlsx</xltc:text>
+    <xltc:text>Источник: photo_4_plantar_pretest3_2026-07-14.xlsx</xltc:text>
   </xltc:threadedComment>
   <xltc:threadedComment ref="A6" dT="2026-09-14T15:06:57.547" personId="{B425DE92-BFBD-455F-8ACE-961BDAB0B5C7}" id="{7E198E70-76D5-477E-9BC0-F02E78DC8B3E}">
-    <xltc:text>Sequential ID. The ROW()-6 formula updates numbering when data rows are inserted or deleted.</xltc:text>
+    <xltc:text>Порядковый номер. Формула ROW()-6 пересчитывает нумерацию при вставке и удалении строк данных.</xltc:text>
   </xltc:threadedComment>
   <xltc:threadedComment ref="B6" dT="2026-09-14T15:06:57.547" personId="{B425DE92-BFBD-455F-8ACE-961BDAB0B5C7}" id="{2BB9EF0D-B28B-4540-92A9-842AB15BB924}">
-    <xltc:text>L1: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</xltc:text>
+    <xltc:text>L1: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</xltc:text>
   </xltc:threadedComment>
   <xltc:threadedComment ref="C6" dT="2026-09-14T15:06:57.547" personId="{B425DE92-BFBD-455F-8ACE-961BDAB0B5C7}" id="{D62184AA-88C1-4ECB-A0BD-0891D8D89FB3}">
-    <xltc:text>L2: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</xltc:text>
+    <xltc:text>L2: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</xltc:text>
   </xltc:threadedComment>
   <xltc:threadedComment ref="D6" dT="2026-09-14T15:06:57.547" personId="{B425DE92-BFBD-455F-8ACE-961BDAB0B5C7}" id="{C2287B28-B146-4551-86FE-13E25228AE0E}">
-    <xltc:text>L3: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</xltc:text>
+    <xltc:text>L3: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</xltc:text>
   </xltc:threadedComment>
   <xltc:threadedComment ref="E6" dT="2026-09-14T15:06:57.547" personId="{B425DE92-BFBD-455F-8ACE-961BDAB0B5C7}" id="{D268E280-C847-4118-8F04-EF7BEA6A93FB}">
-    <xltc:text>L4: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</xltc:text>
+    <xltc:text>L4: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</xltc:text>
   </xltc:threadedComment>
   <xltc:threadedComment ref="F6" dT="2026-09-14T15:06:57.547" personId="{B425DE92-BFBD-455F-8ACE-961BDAB0B5C7}" id="{9023BB59-D0CA-4804-A401-84BBEAD202FB}">
-    <xltc:text>L5: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</xltc:text>
+    <xltc:text>L5: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</xltc:text>
   </xltc:threadedComment>
   <xltc:threadedComment ref="G6" dT="2026-09-14T15:06:57.547" personId="{B425DE92-BFBD-455F-8ACE-961BDAB0B5C7}" id="{BBF23496-A979-4DAE-900E-44836F3969BD}">
-    <xltc:text>R1: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</xltc:text>
+    <xltc:text>R1: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</xltc:text>
   </xltc:threadedComment>
   <xltc:threadedComment ref="H6" dT="2026-09-14T15:06:57.547" personId="{B425DE92-BFBD-455F-8ACE-961BDAB0B5C7}" id="{B1E53955-7046-4945-B67D-B3A8B10C7DCA}">
-    <xltc:text>R2: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</xltc:text>
+    <xltc:text>R2: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</xltc:text>
   </xltc:threadedComment>
   <xltc:threadedComment ref="I6" dT="2026-09-14T15:06:57.547" personId="{B425DE92-BFBD-455F-8ACE-961BDAB0B5C7}" id="{0F6FD458-6F5C-436B-A59C-C20E7FC20B57}">
-    <xltc:text>R3: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</xltc:text>
+    <xltc:text>R3: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</xltc:text>
   </xltc:threadedComment>
   <xltc:threadedComment ref="J6" dT="2026-09-14T15:06:57.547" personId="{B425DE92-BFBD-455F-8ACE-961BDAB0B5C7}" id="{D4C82D69-41FB-4112-A336-1E959AFC68DD}">
-    <xltc:text>R4: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</xltc:text>
+    <xltc:text>R4: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</xltc:text>
   </xltc:threadedComment>
   <xltc:threadedComment ref="K6" dT="2026-09-14T15:06:57.547" personId="{B425DE92-BFBD-455F-8ACE-961BDAB0B5C7}" id="{E82F6BD1-90E0-4943-9F3E-3B50C72A69DA}">
-    <xltc:text>R5: nonnegative number. A blank cell means missing data, not zero. This rule covers every data row.</xltc:text>
+    <xltc:text>R5: неотрицательное число. Пустая клетка означает пропуск, не ноль. Правило применяется ко всем строкам данных.</xltc:text>
   </xltc:threadedComment>
   <xltc:threadedComment ref="L6" dT="2026-09-14T15:06:57.547" personId="{B425DE92-BFBD-455F-8ACE-961BDAB0B5C7}" id="{3EF98C35-30F7-4075-A839-EC8649223C9E}">
-    <xltc:text>Animal notes; recognized and exported as text.</xltc:text>
+    <xltc:text>Примечание к животному; переносится как текст.</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <pageSetUpPr fitToPage="1" autoPageBreaks="0"/>
   </sheetPr>
@@ -617,38 +694,38 @@
       <c r="L2" s="1"/>
     </row>
     <row r="3" ht="13" customHeight="1">
-      <c r="A3" s="3" t="str">
+      <c r="A3" s="28" t="str">
         <v>Date</v>
       </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="3" t="str">
+      <c r="B3" s="29"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="28" t="str">
         <v>Session</v>
       </c>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="3" t="str">
+      <c r="E3" s="29"/>
+      <c r="F3" s="30"/>
+      <c r="G3" s="28" t="str">
         <v>Operator</v>
       </c>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
-      <c r="L3" s="1"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="30"/>
+      <c r="J3"/>
+      <c r="K3"/>
+      <c r="L3"/>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
+      <c r="A4" s="31"/>
+      <c r="B4" s="32"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="31"/>
+      <c r="E4" s="32"/>
+      <c r="F4" s="33"/>
+      <c r="G4" s="31"/>
+      <c r="H4" s="32"/>
+      <c r="I4" s="33"/>
+      <c r="J4"/>
+      <c r="K4"/>
+      <c r="L4"/>
     </row>
     <row r="5" ht="8" customHeight="1">
       <c r="A5" s="1"/>
@@ -1049,16 +1126,16 @@
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="D3:F3"/>
     <mergeCell ref="D4:F4"/>
-    <mergeCell ref="G3:L3"/>
-    <mergeCell ref="G4:L4"/>
+    <mergeCell ref="G3:I3"/>
+    <mergeCell ref="G4:I4"/>
   </mergeCells>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.3937" right="0.3937" top="0.3937" bottom="0.3937" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="1" horizontalDpi="0" verticalDpi="0"/>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <headerFooter/>
-  <legacyDrawing r:id="Re817fee3380a4761"/>
+  <legacyDrawing ns1:id="Rc3d026b6e71942ca"/>
   <tableParts count="1">
-    <tablePart r:id="R66327220f0c8425b"/>
+    <tablePart ns1:id="R2b009867eab2409a"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>